<commit_message>
update 1 in the experiment running
</commit_message>
<xml_diff>
--- a/logs/hypothesis_reinjection_results/experiments_summary.xlsx
+++ b/logs/hypothesis_reinjection_results/experiments_summary.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BW4"/>
+  <dimension ref="A1:BW16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1356,11 +1356,7 @@
       <c r="F4" t="n">
         <v>16590</v>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>['wv', 'sv', 'yr', 'ya', 'rarad']</t>
@@ -1425,10 +1421,8 @@
           <t>lin</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="V4" t="n">
+        <v>1</v>
       </c>
       <c r="W4" t="inlineStr">
         <is>
@@ -1596,6 +1590,3164 @@
       </c>
       <c r="BW4" t="n">
         <v>-0.004729700248401025</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>46080.42480324074</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>02-27_10-11-43_multihead_spsa_compact_f5_w5_h5_effsu2_lin_r1.pkl</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Best (Lowest Val Loss)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>data/reduce_row_number_absolutes</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>16590</v>
+      </c>
+      <c r="G5" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>['wv', 'sv', 'yr', 'ya', 'rarad']</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>['Surge Velocity', 'Sway Velocity', 'Yaw Rate', 'Yaw Angle']</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K5" t="n">
+        <v>5</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>motion</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>multihead</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>[{'features': ['wv', 'sv', 'yr', 'ya', 'rarad'], 'output_dim': 4, 'reps': 1, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [0, 3, -1, 0, 1, 2, 0, -1, 4]}]</t>
+        </is>
+      </c>
+      <c r="R5" t="n">
+        <v>1</v>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>compact</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>effsu2</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>lin</t>
+        </is>
+      </c>
+      <c r="V5" t="n">
+        <v>1</v>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>[0, 3, -1, 0, 1, 2, 0, -1, 4]</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>spsa</t>
+        </is>
+      </c>
+      <c r="Z5" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="n">
+        <v>512</v>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>[0.05, 0.001]</t>
+        </is>
+      </c>
+      <c r="AE5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>130</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>10</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>120</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>0.2451072041504313</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>84.10595742748717</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>0.1962242619145765</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>-1.054989161822768</v>
+      </c>
+      <c r="AM5" t="n">
+        <v>89.66609035405342</v>
+      </c>
+      <c r="AN5" t="n">
+        <v>0.2082910753701545</v>
+      </c>
+      <c r="AO5" t="n">
+        <v>89.66609035405342</v>
+      </c>
+      <c r="AP5" t="n">
+        <v>89.66609035405342</v>
+      </c>
+      <c r="AQ5" t="n">
+        <v>0.2082910753701545</v>
+      </c>
+      <c r="AR5" t="n">
+        <v>90.23417620246045</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>-0.6167791613229727</v>
+      </c>
+      <c r="AT5" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AU5" t="inlineStr">
+        <is>
+          <t>identity</t>
+        </is>
+      </c>
+      <c r="AV5" t="n">
+        <v>0.01932173911105154</v>
+      </c>
+      <c r="AW5" t="n">
+        <v>0.8596991918462569</v>
+      </c>
+      <c r="AX5" t="n">
+        <v>0.01932173911105154</v>
+      </c>
+      <c r="AY5" t="n">
+        <v>0.01932173911105154</v>
+      </c>
+      <c r="AZ5" t="n">
+        <v>0.8596991918462569</v>
+      </c>
+      <c r="BA5" t="n">
+        <v>0.4718182791720155</v>
+      </c>
+      <c r="BB5" t="n">
+        <v>-2.426010748260205</v>
+      </c>
+      <c r="BC5" t="n">
+        <v>0.2894655474110302</v>
+      </c>
+      <c r="BD5" t="n">
+        <v>-0.002936297145538447</v>
+      </c>
+      <c r="BE5" t="n">
+        <v>0.2894655474110302</v>
+      </c>
+      <c r="BF5" t="n">
+        <v>0.2894655474110302</v>
+      </c>
+      <c r="BG5" t="n">
+        <v>-0.002936297145538447</v>
+      </c>
+      <c r="BH5" t="n">
+        <v>0.2923274833639927</v>
+      </c>
+      <c r="BI5" t="n">
+        <v>-0.0128522939645177</v>
+      </c>
+      <c r="BJ5" t="n">
+        <v>0.2501735060302632</v>
+      </c>
+      <c r="BK5" t="n">
+        <v>-0.00436749635500866</v>
+      </c>
+      <c r="BL5" t="n">
+        <v>0.2501735060302632</v>
+      </c>
+      <c r="BM5" t="n">
+        <v>0.2501735060302632</v>
+      </c>
+      <c r="BN5" t="n">
+        <v>-0.00436749635500866</v>
+      </c>
+      <c r="BO5" t="n">
+        <v>0.2500447746140236</v>
+      </c>
+      <c r="BP5" t="n">
+        <v>-0.003850680436798593</v>
+      </c>
+      <c r="BQ5" t="n">
+        <v>358.1054006236609</v>
+      </c>
+      <c r="BR5" t="n">
+        <v>-0.01923109686509572</v>
+      </c>
+      <c r="BS5" t="n">
+        <v>358.1054006236609</v>
+      </c>
+      <c r="BT5" t="n">
+        <v>358.1054006236609</v>
+      </c>
+      <c r="BU5" t="n">
+        <v>-0.01923109686509572</v>
+      </c>
+      <c r="BV5" t="n">
+        <v>359.9225142726907</v>
+      </c>
+      <c r="BW5" t="n">
+        <v>-0.02440292263036947</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>46080.53836805555</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>02-27_12-55-15_multihead_spsa_compact_f5_w5_h5_effsu2_lin_r1.pkl</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Best (Lowest Val Loss)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>data/reduce_row_number_absolutes</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>16590</v>
+      </c>
+      <c r="G6" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>['wv', 'sv', 'yr', 'ya', 'rarad']</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>['Surge Velocity', 'Sway Velocity', 'Yaw Rate', 'Yaw Angle']</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>5</v>
+      </c>
+      <c r="K6" t="n">
+        <v>5</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>motion</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>multihead</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>[{'features': ['wv', 'sv', 'yr', 'ya', 'rarad'], 'output_dim': 4, 'reps': 1, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [0, 3, -1, 0, 1, 2, 0, -1, 4]}]</t>
+        </is>
+      </c>
+      <c r="R6" t="n">
+        <v>1</v>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>compact</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>effsu2</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>lin</t>
+        </is>
+      </c>
+      <c r="V6" t="n">
+        <v>1</v>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>[0, 3, -1, 0, 1, 2, 0, -1, 4]</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>spsa</t>
+        </is>
+      </c>
+      <c r="Z6" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="n">
+        <v>512</v>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>[0.05, 0.001]</t>
+        </is>
+      </c>
+      <c r="AE6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>130</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>10</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>120</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>0.2528091430146155</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>83.45153897521642</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>0.1952558855820531</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>-1.088189862519791</v>
+      </c>
+      <c r="AM6" t="n">
+        <v>89.23345334154796</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>0.2068035630998364</v>
+      </c>
+      <c r="AO6" t="n">
+        <v>89.23345334154796</v>
+      </c>
+      <c r="AP6" t="n">
+        <v>89.23345334154796</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>0.2068035630998364</v>
+      </c>
+      <c r="AR6" t="n">
+        <v>89.74249513825836</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>-0.6357547323465322</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AU6" t="inlineStr">
+        <is>
+          <t>identity</t>
+        </is>
+      </c>
+      <c r="AV6" t="n">
+        <v>0.02060162159461616</v>
+      </c>
+      <c r="AW6" t="n">
+        <v>0.8504055901805959</v>
+      </c>
+      <c r="AX6" t="n">
+        <v>0.02060162159461616</v>
+      </c>
+      <c r="AY6" t="n">
+        <v>0.02060162159461616</v>
+      </c>
+      <c r="AZ6" t="n">
+        <v>0.8504055901805959</v>
+      </c>
+      <c r="BA6" t="n">
+        <v>0.4815339366522431</v>
+      </c>
+      <c r="BB6" t="n">
+        <v>-2.496558983508927</v>
+      </c>
+      <c r="BC6" t="n">
+        <v>0.2885836957922676</v>
+      </c>
+      <c r="BD6" t="n">
+        <v>0.0001191303658318876</v>
+      </c>
+      <c r="BE6" t="n">
+        <v>0.2885836957922676</v>
+      </c>
+      <c r="BF6" t="n">
+        <v>0.2885836957922676</v>
+      </c>
+      <c r="BG6" t="n">
+        <v>0.0001191303658318876</v>
+      </c>
+      <c r="BH6" t="n">
+        <v>0.2945397089979261</v>
+      </c>
+      <c r="BI6" t="n">
+        <v>-0.0205171832944977</v>
+      </c>
+      <c r="BJ6" t="n">
+        <v>0.2513296975705513</v>
+      </c>
+      <c r="BK6" t="n">
+        <v>-0.009009239683678949</v>
+      </c>
+      <c r="BL6" t="n">
+        <v>0.2513296975705513</v>
+      </c>
+      <c r="BM6" t="n">
+        <v>0.2513296975705513</v>
+      </c>
+      <c r="BN6" t="n">
+        <v>-0.009009239683678949</v>
+      </c>
+      <c r="BO6" t="n">
+        <v>0.2508725130963913</v>
+      </c>
+      <c r="BP6" t="n">
+        <v>-0.007173788628246358</v>
+      </c>
+      <c r="BQ6" t="n">
+        <v>356.3732983512335</v>
+      </c>
+      <c r="BR6" t="n">
+        <v>-0.01430122846340698</v>
+      </c>
+      <c r="BS6" t="n">
+        <v>356.3732983512335</v>
+      </c>
+      <c r="BT6" t="n">
+        <v>356.3732983512335</v>
+      </c>
+      <c r="BU6" t="n">
+        <v>-0.01430122846340698</v>
+      </c>
+      <c r="BV6" t="n">
+        <v>357.943034394287</v>
+      </c>
+      <c r="BW6" t="n">
+        <v>-0.01876897395443744</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>46080.64230324074</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>02-27_15-24-55_multihead_spsa_compact_f5_w5_h5_effsu2_lin_r1.pkl</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Best (Lowest Val Loss)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>data/reduce_row_number_absolutes</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>16590</v>
+      </c>
+      <c r="G7" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>['wv', 'sv', 'yr', 'ya', 'rarad']</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>['Surge Velocity', 'Sway Velocity', 'Yaw Rate', 'Yaw Angle']</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>5</v>
+      </c>
+      <c r="K7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>motion</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>multihead</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>[{'features': ['wv', 'sv', 'yr', 'ya', 'rarad'], 'output_dim': 4, 'reps': 1, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [0, 3, -1, 0, 1, 2, 0, -1, 4]}]</t>
+        </is>
+      </c>
+      <c r="R7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>compact</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>effsu2</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>lin</t>
+        </is>
+      </c>
+      <c r="V7" t="n">
+        <v>1</v>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>[0, 3, -1, 0, 1, 2, 0, -1, 4]</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>spsa</t>
+        </is>
+      </c>
+      <c r="Z7" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="n">
+        <v>512</v>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>[0.05, 0.001]</t>
+        </is>
+      </c>
+      <c r="AE7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>130</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>10</v>
+      </c>
+      <c r="AH7" t="n">
+        <v>120</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>0.247709079131496</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>83.99654957183179</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>0.1960658241128452</v>
+      </c>
+      <c r="AL7" t="n">
+        <v>-1.241819633039339</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>89.53400874820487</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>0.2073074242219778</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>89.53400874820487</v>
+      </c>
+      <c r="AP7" t="n">
+        <v>89.53400874820487</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>0.2073074242219778</v>
+      </c>
+      <c r="AR7" t="n">
+        <v>89.96088791523681</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>-0.7220707257890304</v>
+      </c>
+      <c r="AT7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AU7" t="inlineStr">
+        <is>
+          <t>identity</t>
+        </is>
+      </c>
+      <c r="AV7" t="n">
+        <v>0.01990834430042695</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>0.8554396797152047</v>
+      </c>
+      <c r="AX7" t="n">
+        <v>0.01990834430042695</v>
+      </c>
+      <c r="AY7" t="n">
+        <v>0.01990834430042695</v>
+      </c>
+      <c r="AZ7" t="n">
+        <v>0.8554396797152047</v>
+      </c>
+      <c r="BA7" t="n">
+        <v>0.5278932700357961</v>
+      </c>
+      <c r="BB7" t="n">
+        <v>-2.833187684569331</v>
+      </c>
+      <c r="BC7" t="n">
+        <v>0.2902156842770169</v>
+      </c>
+      <c r="BD7" t="n">
+        <v>-0.005535361170442066</v>
+      </c>
+      <c r="BE7" t="n">
+        <v>0.2902156842770169</v>
+      </c>
+      <c r="BF7" t="n">
+        <v>0.2902156842770169</v>
+      </c>
+      <c r="BG7" t="n">
+        <v>-0.005535361170442066</v>
+      </c>
+      <c r="BH7" t="n">
+        <v>0.2923525619231196</v>
+      </c>
+      <c r="BI7" t="n">
+        <v>-0.01293918581556319</v>
+      </c>
+      <c r="BJ7" t="n">
+        <v>0.2498204366903786</v>
+      </c>
+      <c r="BK7" t="n">
+        <v>-0.002950034631876486</v>
+      </c>
+      <c r="BL7" t="n">
+        <v>0.2498204366903786</v>
+      </c>
+      <c r="BM7" t="n">
+        <v>0.2498204366903786</v>
+      </c>
+      <c r="BN7" t="n">
+        <v>-0.002950034631876486</v>
+      </c>
+      <c r="BO7" t="n">
+        <v>0.2543254581810783</v>
+      </c>
+      <c r="BP7" t="n">
+        <v>-0.02103627097015703</v>
+      </c>
+      <c r="BQ7" t="n">
+        <v>357.5760905275494</v>
+      </c>
+      <c r="BR7" t="n">
+        <v>-0.01772458702497048</v>
+      </c>
+      <c r="BS7" t="n">
+        <v>357.5760905275494</v>
+      </c>
+      <c r="BT7" t="n">
+        <v>357.5760905275494</v>
+      </c>
+      <c r="BU7" t="n">
+        <v>-0.01772458702497048</v>
+      </c>
+      <c r="BV7" t="n">
+        <v>358.7689803708087</v>
+      </c>
+      <c r="BW7" t="n">
+        <v>-0.02111976180107544</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>46080.74046296296</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>02-27_17-46-16_multihead_spsa_compact_f5_w5_h5_effsu2_lin_r1.pkl</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Best (Lowest Val Loss)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>data/reduce_row_number_absolutes</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>16590</v>
+      </c>
+      <c r="G8" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>['wv', 'sv', 'yr', 'ya', 'rarad']</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>['Surge Velocity', 'Sway Velocity', 'Yaw Rate', 'Yaw Angle']</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>5</v>
+      </c>
+      <c r="K8" t="n">
+        <v>5</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>motion</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>multihead</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>[{'features': ['wv', 'sv', 'yr', 'ya', 'rarad'], 'output_dim': 4, 'reps': 1, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [0, 1, -1, 2, 3, -1, 0, 2, 4]}]</t>
+        </is>
+      </c>
+      <c r="R8" t="n">
+        <v>1</v>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>compact</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>effsu2</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>lin</t>
+        </is>
+      </c>
+      <c r="V8" t="n">
+        <v>1</v>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>[0, 1, -1, 2, 3, -1, 0, 2, 4]</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>spsa</t>
+        </is>
+      </c>
+      <c r="Z8" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="n">
+        <v>512</v>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>[0.05, 0.001]</t>
+        </is>
+      </c>
+      <c r="AE8" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>130</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>10</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>120</v>
+      </c>
+      <c r="AI8" t="n">
+        <v>0.1873464741731447</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>61.97975757851797</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>0.3181734018552846</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>-1.408393343248677</v>
+      </c>
+      <c r="AM8" t="n">
+        <v>69.59437522802411</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>0.3375376824637001</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>69.59437522802411</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>69.59437522802411</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>0.3375376824637001</v>
+      </c>
+      <c r="AR8" t="n">
+        <v>207.1867426279353</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>-1.098569254452363</v>
+      </c>
+      <c r="AT8" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AU8" t="inlineStr">
+        <is>
+          <t>identity</t>
+        </is>
+      </c>
+      <c r="AV8" t="n">
+        <v>0.09557331346604735</v>
+      </c>
+      <c r="AW8" t="n">
+        <v>0.3060141719050616</v>
+      </c>
+      <c r="AX8" t="n">
+        <v>0.09557331346604735</v>
+      </c>
+      <c r="AY8" t="n">
+        <v>0.09557331346604735</v>
+      </c>
+      <c r="AZ8" t="n">
+        <v>0.3060141719050616</v>
+      </c>
+      <c r="BA8" t="n">
+        <v>0.401086790115408</v>
+      </c>
+      <c r="BB8" t="n">
+        <v>-1.912408684826714</v>
+      </c>
+      <c r="BC8" t="n">
+        <v>0.1476112868217098</v>
+      </c>
+      <c r="BD8" t="n">
+        <v>0.4885584182782358</v>
+      </c>
+      <c r="BE8" t="n">
+        <v>0.1476112868217098</v>
+      </c>
+      <c r="BF8" t="n">
+        <v>0.1476112868217098</v>
+      </c>
+      <c r="BG8" t="n">
+        <v>0.4885584182782358</v>
+      </c>
+      <c r="BH8" t="n">
+        <v>0.5124042794409541</v>
+      </c>
+      <c r="BI8" t="n">
+        <v>-0.7753713879265465</v>
+      </c>
+      <c r="BJ8" t="n">
+        <v>0.1627190939660126</v>
+      </c>
+      <c r="BK8" t="n">
+        <v>0.346734306085835</v>
+      </c>
+      <c r="BL8" t="n">
+        <v>0.1627190939660126</v>
+      </c>
+      <c r="BM8" t="n">
+        <v>0.1627190939660126</v>
+      </c>
+      <c r="BN8" t="n">
+        <v>0.346734306085835</v>
+      </c>
+      <c r="BO8" t="n">
+        <v>0.3365881407298638</v>
+      </c>
+      <c r="BP8" t="n">
+        <v>-0.3512949215603431</v>
+      </c>
+      <c r="BQ8" t="n">
+        <v>277.9715972178436</v>
+      </c>
+      <c r="BR8" t="n">
+        <v>0.2088438335856645</v>
+      </c>
+      <c r="BS8" t="n">
+        <v>277.9715972178436</v>
+      </c>
+      <c r="BT8" t="n">
+        <v>277.9715972178436</v>
+      </c>
+      <c r="BU8" t="n">
+        <v>0.2088438335856645</v>
+      </c>
+      <c r="BV8" t="n">
+        <v>827.4968913014584</v>
+      </c>
+      <c r="BW8" t="n">
+        <v>-1.355202023495861</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>46080.83997685185</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>02-27_20-09-34_multihead_spsa_compact_f5_w5_h5_effsu2_lin_r1.pkl</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Best (Lowest Val Loss)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>data/reduce_row_number_absolutes</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>16590</v>
+      </c>
+      <c r="G9" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>['wv', 'sv', 'yr', 'ya', 'rarad']</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>['Surge Velocity', 'Sway Velocity', 'Yaw Rate', 'Yaw Angle']</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>5</v>
+      </c>
+      <c r="K9" t="n">
+        <v>5</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>motion</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>multihead</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>[{'features': ['wv', 'sv', 'yr', 'ya', 'rarad'], 'output_dim': 4, 'reps': 1, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [0, 1, -1, 2, 3, -1, 0, 2, 4]}]</t>
+        </is>
+      </c>
+      <c r="R9" t="n">
+        <v>1</v>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>compact</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>effsu2</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>lin</t>
+        </is>
+      </c>
+      <c r="V9" t="n">
+        <v>1</v>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>[0, 1, -1, 2, 3, -1, 0, 2, 4]</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>spsa</t>
+        </is>
+      </c>
+      <c r="Z9" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="n">
+        <v>512</v>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>[0.05, 0.001]</t>
+        </is>
+      </c>
+      <c r="AE9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>130</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>10</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>120</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>0.1965043831768628</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>62.0752205166223</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>0.3095818089369431</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>-1.330260000683264</v>
+      </c>
+      <c r="AM9" t="n">
+        <v>69.71356878947833</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>0.330091459161864</v>
+      </c>
+      <c r="AO9" t="n">
+        <v>69.71356878947833</v>
+      </c>
+      <c r="AP9" t="n">
+        <v>69.71356878947833</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>0.330091459161864</v>
+      </c>
+      <c r="AR9" t="n">
+        <v>184.9331272125302</v>
+      </c>
+      <c r="AS9" t="n">
+        <v>-1.04879965118946</v>
+      </c>
+      <c r="AT9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AU9" t="inlineStr">
+        <is>
+          <t>identity</t>
+        </is>
+      </c>
+      <c r="AV9" t="n">
+        <v>0.0985168960239633</v>
+      </c>
+      <c r="AW9" t="n">
+        <v>0.284639956604398</v>
+      </c>
+      <c r="AX9" t="n">
+        <v>0.0985168960239633</v>
+      </c>
+      <c r="AY9" t="n">
+        <v>0.0985168960239633</v>
+      </c>
+      <c r="AZ9" t="n">
+        <v>0.284639956604398</v>
+      </c>
+      <c r="BA9" t="n">
+        <v>0.4061938973979063</v>
+      </c>
+      <c r="BB9" t="n">
+        <v>-1.949492886975605</v>
+      </c>
+      <c r="BC9" t="n">
+        <v>0.1483699278075956</v>
+      </c>
+      <c r="BD9" t="n">
+        <v>0.4859298892942089</v>
+      </c>
+      <c r="BE9" t="n">
+        <v>0.1483699278075956</v>
+      </c>
+      <c r="BF9" t="n">
+        <v>0.1483699278075956</v>
+      </c>
+      <c r="BG9" t="n">
+        <v>0.4859298892942089</v>
+      </c>
+      <c r="BH9" t="n">
+        <v>0.5291956259737324</v>
+      </c>
+      <c r="BI9" t="n">
+        <v>-0.8335498173330662</v>
+      </c>
+      <c r="BJ9" t="n">
+        <v>0.1638247475549674</v>
+      </c>
+      <c r="BK9" t="n">
+        <v>0.3422954566465176</v>
+      </c>
+      <c r="BL9" t="n">
+        <v>0.1638247475549674</v>
+      </c>
+      <c r="BM9" t="n">
+        <v>0.1638247475549674</v>
+      </c>
+      <c r="BN9" t="n">
+        <v>0.3422954566465176</v>
+      </c>
+      <c r="BO9" t="n">
+        <v>0.3263863645615373</v>
+      </c>
+      <c r="BP9" t="n">
+        <v>-0.3103380170857473</v>
+      </c>
+      <c r="BQ9" t="n">
+        <v>278.443563586527</v>
+      </c>
+      <c r="BR9" t="n">
+        <v>0.2075005341023314</v>
+      </c>
+      <c r="BS9" t="n">
+        <v>278.443563586527</v>
+      </c>
+      <c r="BT9" t="n">
+        <v>278.443563586527</v>
+      </c>
+      <c r="BU9" t="n">
+        <v>0.2075005341023314</v>
+      </c>
+      <c r="BV9" t="n">
+        <v>738.470732962185</v>
+      </c>
+      <c r="BW9" t="n">
+        <v>-1.101817883363382</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>46080.93869212963</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>02-27_22-31-43_multihead_spsa_compact_f5_w5_h5_effsu2_lin_r1.pkl</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Final (Last Iteration)</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>data/reduce_row_number_absolutes</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>16590</v>
+      </c>
+      <c r="G10" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>['wv', 'sv', 'yr', 'ya', 'rarad']</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>['Surge Velocity', 'Sway Velocity', 'Yaw Rate', 'Yaw Angle']</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>5</v>
+      </c>
+      <c r="K10" t="n">
+        <v>5</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>motion</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>multihead</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>[{'features': ['wv', 'sv', 'yr', 'ya', 'rarad'], 'output_dim': 4, 'reps': 1, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [0, 1, -1, 2, 3, -1, 0, 2, 4]}]</t>
+        </is>
+      </c>
+      <c r="R10" t="n">
+        <v>1</v>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>compact</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>effsu2</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>lin</t>
+        </is>
+      </c>
+      <c r="V10" t="n">
+        <v>1</v>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>[0, 1, -1, 2, 3, -1, 0, 2, 4]</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>spsa</t>
+        </is>
+      </c>
+      <c r="Z10" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="n">
+        <v>512</v>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>[0.05, 0.001]</t>
+        </is>
+      </c>
+      <c r="AE10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>130</v>
+      </c>
+      <c r="AG10" t="n">
+        <v>10</v>
+      </c>
+      <c r="AH10" t="n">
+        <v>120</v>
+      </c>
+      <c r="AI10" t="n">
+        <v>0.1914015653522703</v>
+      </c>
+      <c r="AJ10" t="n">
+        <v>61.99888895761318</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>0.3163179108295318</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>-1.559459225680615</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>69.66717254116332</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>0.3363325895848371</v>
+      </c>
+      <c r="AO10" t="n">
+        <v>69.66717254116332</v>
+      </c>
+      <c r="AP10" t="n">
+        <v>69.66717254116332</v>
+      </c>
+      <c r="AQ10" t="n">
+        <v>0.3363325895848371</v>
+      </c>
+      <c r="AR10" t="n">
+        <v>190.1097210386185</v>
+      </c>
+      <c r="AS10" t="n">
+        <v>-1.059487066887807</v>
+      </c>
+      <c r="AT10" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AU10" t="inlineStr">
+        <is>
+          <t>identity</t>
+        </is>
+      </c>
+      <c r="AV10" t="n">
+        <v>0.09344128237194173</v>
+      </c>
+      <c r="AW10" t="n">
+        <v>0.3214954742760699</v>
+      </c>
+      <c r="AX10" t="n">
+        <v>0.09344128237194173</v>
+      </c>
+      <c r="AY10" t="n">
+        <v>0.09344128237194173</v>
+      </c>
+      <c r="AZ10" t="n">
+        <v>0.3214954742760699</v>
+      </c>
+      <c r="BA10" t="n">
+        <v>0.4303743527247104</v>
+      </c>
+      <c r="BB10" t="n">
+        <v>-2.125074256974315</v>
+      </c>
+      <c r="BC10" t="n">
+        <v>0.1506665948059113</v>
+      </c>
+      <c r="BD10" t="n">
+        <v>0.4779724286718006</v>
+      </c>
+      <c r="BE10" t="n">
+        <v>0.1506665948059113</v>
+      </c>
+      <c r="BF10" t="n">
+        <v>0.1506665948059113</v>
+      </c>
+      <c r="BG10" t="n">
+        <v>0.4779724286718006</v>
+      </c>
+      <c r="BH10" t="n">
+        <v>0.4740916294452314</v>
+      </c>
+      <c r="BI10" t="n">
+        <v>-0.6426262385841932</v>
+      </c>
+      <c r="BJ10" t="n">
+        <v>0.164934920528517</v>
+      </c>
+      <c r="BK10" t="n">
+        <v>0.3378384633075423</v>
+      </c>
+      <c r="BL10" t="n">
+        <v>0.164934920528517</v>
+      </c>
+      <c r="BM10" t="n">
+        <v>0.164934920528517</v>
+      </c>
+      <c r="BN10" t="n">
+        <v>0.3378384633075423</v>
+      </c>
+      <c r="BO10" t="n">
+        <v>0.3261545165544021</v>
+      </c>
+      <c r="BP10" t="n">
+        <v>-0.3094072206710656</v>
+      </c>
+      <c r="BQ10" t="n">
+        <v>278.2596473669464</v>
+      </c>
+      <c r="BR10" t="n">
+        <v>0.2080239920839424</v>
+      </c>
+      <c r="BS10" t="n">
+        <v>278.2596473669464</v>
+      </c>
+      <c r="BT10" t="n">
+        <v>278.2596473669464</v>
+      </c>
+      <c r="BU10" t="n">
+        <v>0.2080239920839424</v>
+      </c>
+      <c r="BV10" t="n">
+        <v>759.2082636557517</v>
+      </c>
+      <c r="BW10" t="n">
+        <v>-1.160840551321663</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>46081.03609953704</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>02-28_00-51-59_multihead_spsa_compact_f5_w5_h5_effsu2_lin_r1.pkl</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Final (Last Iteration)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>data/reduce_row_number_absolutes</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>16590</v>
+      </c>
+      <c r="G11" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>['wv', 'sv', 'yr', 'ya', 'rarad']</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>['Surge Velocity', 'Sway Velocity', 'Yaw Rate', 'Yaw Angle']</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>5</v>
+      </c>
+      <c r="K11" t="n">
+        <v>5</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>motion</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>multihead</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>[{'features': ['wv', 'sv', 'yr', 'ya', 'rarad'], 'output_dim': 4, 'reps': 1, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [-1, 0, 1, -1, 2, 3, -1, 4, 0]}]</t>
+        </is>
+      </c>
+      <c r="R11" t="n">
+        <v>1</v>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>compact</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>effsu2</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>lin</t>
+        </is>
+      </c>
+      <c r="V11" t="n">
+        <v>1</v>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>[-1, 0, 1, -1, 2, 3, -1, 4, 0]</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>spsa</t>
+        </is>
+      </c>
+      <c r="Z11" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="n">
+        <v>512</v>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>[0.05, 0.001]</t>
+        </is>
+      </c>
+      <c r="AE11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>130</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>10</v>
+      </c>
+      <c r="AH11" t="n">
+        <v>120</v>
+      </c>
+      <c r="AI11" t="n">
+        <v>0.2813172414036672</v>
+      </c>
+      <c r="AJ11" t="n">
+        <v>83.58083645356102</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>-0.02725559539924011</v>
+      </c>
+      <c r="AL11" t="n">
+        <v>-0.02735872919053944</v>
+      </c>
+      <c r="AM11" t="n">
+        <v>88.04894107230125</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>-0.02189650618200006</v>
+      </c>
+      <c r="AO11" t="n">
+        <v>88.04894107230125</v>
+      </c>
+      <c r="AP11" t="n">
+        <v>88.04894107230125</v>
+      </c>
+      <c r="AQ11" t="n">
+        <v>-0.02189650618200006</v>
+      </c>
+      <c r="AR11" t="n">
+        <v>88.0451411414209</v>
+      </c>
+      <c r="AS11" t="n">
+        <v>-0.02182730963826546</v>
+      </c>
+      <c r="AT11" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AU11" t="inlineStr">
+        <is>
+          <t>identity</t>
+        </is>
+      </c>
+      <c r="AV11" t="n">
+        <v>0.14957393590737</v>
+      </c>
+      <c r="AW11" t="n">
+        <v>-0.08610016758466132</v>
+      </c>
+      <c r="AX11" t="n">
+        <v>0.14957393590737</v>
+      </c>
+      <c r="AY11" t="n">
+        <v>0.14957393590737</v>
+      </c>
+      <c r="AZ11" t="n">
+        <v>-0.08610016758466132</v>
+      </c>
+      <c r="BA11" t="n">
+        <v>0.1495693583719624</v>
+      </c>
+      <c r="BB11" t="n">
+        <v>-0.08606692875903899</v>
+      </c>
+      <c r="BC11" t="n">
+        <v>0.2888094125850059</v>
+      </c>
+      <c r="BD11" t="n">
+        <v>-0.0006629301119598363</v>
+      </c>
+      <c r="BE11" t="n">
+        <v>0.2888094125850059</v>
+      </c>
+      <c r="BF11" t="n">
+        <v>0.2888094125850059</v>
+      </c>
+      <c r="BG11" t="n">
+        <v>-0.0006629301119598363</v>
+      </c>
+      <c r="BH11" t="n">
+        <v>0.2887249549272359</v>
+      </c>
+      <c r="BI11" t="n">
+        <v>-0.0003703023664229921</v>
+      </c>
+      <c r="BJ11" t="n">
+        <v>0.2491774424499054</v>
+      </c>
+      <c r="BK11" t="n">
+        <v>-0.0003686161366798224</v>
+      </c>
+      <c r="BL11" t="n">
+        <v>0.2491774424499054</v>
+      </c>
+      <c r="BM11" t="n">
+        <v>0.2491774424499054</v>
+      </c>
+      <c r="BN11" t="n">
+        <v>-0.0003686161366798224</v>
+      </c>
+      <c r="BO11" t="n">
+        <v>0.2492003965397459</v>
+      </c>
+      <c r="BP11" t="n">
+        <v>-0.0004607695469671658</v>
+      </c>
+      <c r="BQ11" t="n">
+        <v>351.5082034982631</v>
+      </c>
+      <c r="BR11" t="n">
+        <v>-0.0004543108946968299</v>
+      </c>
+      <c r="BS11" t="n">
+        <v>351.5082034982631</v>
+      </c>
+      <c r="BT11" t="n">
+        <v>351.5082034982631</v>
+      </c>
+      <c r="BU11" t="n">
+        <v>-0.0004543108946968299</v>
+      </c>
+      <c r="BV11" t="n">
+        <v>351.4930698558439</v>
+      </c>
+      <c r="BW11" t="n">
+        <v>-0.0004112378806186978</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>46081.1312962963</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>02-28_03-09-04_multihead_spsa_compact_f5_w5_h5_effsu2_lin_r1.pkl</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Best (Lowest Val Loss)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>data/reduce_row_number_absolutes</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>16590</v>
+      </c>
+      <c r="G12" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>['wv', 'sv', 'yr', 'ya', 'rarad']</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>['Surge Velocity', 'Sway Velocity', 'Yaw Rate', 'Yaw Angle']</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>5</v>
+      </c>
+      <c r="K12" t="n">
+        <v>5</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>motion</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>multihead</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>[{'features': ['wv', 'sv', 'yr', 'ya', 'rarad'], 'output_dim': 4, 'reps': 1, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [-1, 0, 1, -1, 2, 3, -1, 4, 0]}]</t>
+        </is>
+      </c>
+      <c r="R12" t="n">
+        <v>1</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>compact</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>effsu2</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>lin</t>
+        </is>
+      </c>
+      <c r="V12" t="n">
+        <v>1</v>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>[-1, 0, 1, -1, 2, 3, -1, 4, 0]</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>spsa</t>
+        </is>
+      </c>
+      <c r="Z12" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AB12" t="inlineStr"/>
+      <c r="AC12" t="n">
+        <v>512</v>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>[0.05, 0.001]</t>
+        </is>
+      </c>
+      <c r="AE12" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>130</v>
+      </c>
+      <c r="AG12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AH12" t="n">
+        <v>120</v>
+      </c>
+      <c r="AI12" t="n">
+        <v>0.2979261617442053</v>
+      </c>
+      <c r="AJ12" t="n">
+        <v>83.55517564460813</v>
+      </c>
+      <c r="AK12" t="n">
+        <v>-0.0285929485942954</v>
+      </c>
+      <c r="AL12" t="n">
+        <v>-0.02856003686725084</v>
+      </c>
+      <c r="AM12" t="n">
+        <v>88.0530544523282</v>
+      </c>
+      <c r="AN12" t="n">
+        <v>-0.02270653640258363</v>
+      </c>
+      <c r="AO12" t="n">
+        <v>88.0530544523282</v>
+      </c>
+      <c r="AP12" t="n">
+        <v>88.0530544523282</v>
+      </c>
+      <c r="AQ12" t="n">
+        <v>-0.02270653640258363</v>
+      </c>
+      <c r="AR12" t="n">
+        <v>88.03279152841684</v>
+      </c>
+      <c r="AS12" t="n">
+        <v>-0.02259247620242083</v>
+      </c>
+      <c r="AT12" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AU12" t="inlineStr">
+        <is>
+          <t>identity</t>
+        </is>
+      </c>
+      <c r="AV12" t="n">
+        <v>0.1500851830119374</v>
+      </c>
+      <c r="AW12" t="n">
+        <v>-0.08981248258512875</v>
+      </c>
+      <c r="AX12" t="n">
+        <v>0.1500851830119374</v>
+      </c>
+      <c r="AY12" t="n">
+        <v>0.1500851830119374</v>
+      </c>
+      <c r="AZ12" t="n">
+        <v>-0.08981248258512875</v>
+      </c>
+      <c r="BA12" t="n">
+        <v>0.1500337657001776</v>
+      </c>
+      <c r="BB12" t="n">
+        <v>-0.08943912642130014</v>
+      </c>
+      <c r="BC12" t="n">
+        <v>0.2886298044981169</v>
+      </c>
+      <c r="BD12" t="n">
+        <v>-4.062645194569114e-05</v>
+      </c>
+      <c r="BE12" t="n">
+        <v>0.2886298044981169</v>
+      </c>
+      <c r="BF12" t="n">
+        <v>0.2886298044981169</v>
+      </c>
+      <c r="BG12" t="n">
+        <v>-4.062645194569114e-05</v>
+      </c>
+      <c r="BH12" t="n">
+        <v>0.2887029149808519</v>
+      </c>
+      <c r="BI12" t="n">
+        <v>-0.0002939386595386395</v>
+      </c>
+      <c r="BJ12" t="n">
+        <v>0.249203421524528</v>
+      </c>
+      <c r="BK12" t="n">
+        <v>-0.0004729139040589025</v>
+      </c>
+      <c r="BL12" t="n">
+        <v>0.249203421524528</v>
+      </c>
+      <c r="BM12" t="n">
+        <v>0.249203421524528</v>
+      </c>
+      <c r="BN12" t="n">
+        <v>-0.0004729139040589025</v>
+      </c>
+      <c r="BO12" t="n">
+        <v>0.2491771373872224</v>
+      </c>
+      <c r="BP12" t="n">
+        <v>-0.0003673914064994399</v>
+      </c>
+      <c r="BQ12" t="n">
+        <v>351.5242994002774</v>
+      </c>
+      <c r="BR12" t="n">
+        <v>-0.0005001226692091798</v>
+      </c>
+      <c r="BS12" t="n">
+        <v>351.5242994002774</v>
+      </c>
+      <c r="BT12" t="n">
+        <v>351.5242994002774</v>
+      </c>
+      <c r="BU12" t="n">
+        <v>-0.0005001226692091798</v>
+      </c>
+      <c r="BV12" t="n">
+        <v>351.4432522955992</v>
+      </c>
+      <c r="BW12" t="n">
+        <v>-0.0002694483223406596</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>46081.21648148148</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>02-28_05-11-44_multihead_spsa_compact_f5_w5_h5_effsu2_lin_r1.pkl</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Best (Lowest Val Loss)</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>data/reduce_row_number_absolutes</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>16590</v>
+      </c>
+      <c r="G13" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>['wv', 'sv', 'yr', 'ya', 'rarad']</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>['Surge Velocity', 'Sway Velocity', 'Yaw Rate', 'Yaw Angle']</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>5</v>
+      </c>
+      <c r="K13" t="n">
+        <v>5</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>motion</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>multihead</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>[{'features': ['wv', 'sv', 'yr', 'ya', 'rarad'], 'output_dim': 4, 'reps': 1, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [-1, 0, 1, -1, 2, 3, -1, 4, 0]}]</t>
+        </is>
+      </c>
+      <c r="R13" t="n">
+        <v>1</v>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>compact</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>effsu2</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>lin</t>
+        </is>
+      </c>
+      <c r="V13" t="n">
+        <v>1</v>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>[-1, 0, 1, -1, 2, 3, -1, 4, 0]</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>spsa</t>
+        </is>
+      </c>
+      <c r="Z13" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AB13" t="inlineStr"/>
+      <c r="AC13" t="n">
+        <v>512</v>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>[0.05, 0.001]</t>
+        </is>
+      </c>
+      <c r="AE13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AF13" t="n">
+        <v>130</v>
+      </c>
+      <c r="AG13" t="n">
+        <v>10</v>
+      </c>
+      <c r="AH13" t="n">
+        <v>120</v>
+      </c>
+      <c r="AI13" t="n">
+        <v>0.2835535920471915</v>
+      </c>
+      <c r="AJ13" t="n">
+        <v>83.56231423555325</v>
+      </c>
+      <c r="AK13" t="n">
+        <v>-0.02809214321828557</v>
+      </c>
+      <c r="AL13" t="n">
+        <v>-0.02848142433038753</v>
+      </c>
+      <c r="AM13" t="n">
+        <v>88.00908797227383</v>
+      </c>
+      <c r="AN13" t="n">
+        <v>-0.02243793735405453</v>
+      </c>
+      <c r="AO13" t="n">
+        <v>88.00908797227383</v>
+      </c>
+      <c r="AP13" t="n">
+        <v>88.00908797227383</v>
+      </c>
+      <c r="AQ13" t="n">
+        <v>-0.02243793735405453</v>
+      </c>
+      <c r="AR13" t="n">
+        <v>87.99675675984757</v>
+      </c>
+      <c r="AS13" t="n">
+        <v>-0.02229947055312664</v>
+      </c>
+      <c r="AT13" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AU13" t="inlineStr">
+        <is>
+          <t>identity</t>
+        </is>
+      </c>
+      <c r="AV13" t="n">
+        <v>0.1499685068676548</v>
+      </c>
+      <c r="AW13" t="n">
+        <v>-0.08896526292022022</v>
+      </c>
+      <c r="AX13" t="n">
+        <v>0.1499685068676548</v>
+      </c>
+      <c r="AY13" t="n">
+        <v>0.1499685068676548</v>
+      </c>
+      <c r="AZ13" t="n">
+        <v>-0.08896526292022022</v>
+      </c>
+      <c r="BA13" t="n">
+        <v>0.1498434906578731</v>
+      </c>
+      <c r="BB13" t="n">
+        <v>-0.08805748359642984</v>
+      </c>
+      <c r="BC13" t="n">
+        <v>0.2887866706792677</v>
+      </c>
+      <c r="BD13" t="n">
+        <v>-0.0005841342658388093</v>
+      </c>
+      <c r="BE13" t="n">
+        <v>0.2887866706792677</v>
+      </c>
+      <c r="BF13" t="n">
+        <v>0.2887866706792677</v>
+      </c>
+      <c r="BG13" t="n">
+        <v>-0.0005841342658388093</v>
+      </c>
+      <c r="BH13" t="n">
+        <v>0.2887866353891007</v>
+      </c>
+      <c r="BI13" t="n">
+        <v>-0.0005840119929474419</v>
+      </c>
+      <c r="BJ13" t="n">
+        <v>0.2491361145752319</v>
+      </c>
+      <c r="BK13" t="n">
+        <v>-0.0002026977919513673</v>
+      </c>
+      <c r="BL13" t="n">
+        <v>0.2491361145752319</v>
+      </c>
+      <c r="BM13" t="n">
+        <v>0.2491361145752319</v>
+      </c>
+      <c r="BN13" t="n">
+        <v>-0.0002026977919513673</v>
+      </c>
+      <c r="BO13" t="n">
+        <v>0.2492592665445991</v>
+      </c>
+      <c r="BP13" t="n">
+        <v>-0.000697113995757892</v>
+      </c>
+      <c r="BQ13" t="n">
+        <v>351.3484605969723</v>
+      </c>
+      <c r="BR13" t="n">
+        <v>3.455617975101077e-07</v>
+      </c>
+      <c r="BS13" t="n">
+        <v>351.3484605969723</v>
+      </c>
+      <c r="BT13" t="n">
+        <v>351.3484605969723</v>
+      </c>
+      <c r="BU13" t="n">
+        <v>3.455617975101077e-07</v>
+      </c>
+      <c r="BV13" t="n">
+        <v>351.2991376467986</v>
+      </c>
+      <c r="BW13" t="n">
+        <v>0.0001407273726236058</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>46081.29846064815</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>02-28_07-09-47_multihead_spsa_compact_f5_w5_h5_effsu2_lin_r1.pkl</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Final (Last Iteration)</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>data/reduce_row_number_absolutes</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>16590</v>
+      </c>
+      <c r="G14" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>['wv', 'sv', 'yr', 'ya', 'rarad']</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>['Surge Velocity', 'Sway Velocity', 'Yaw Rate', 'Yaw Angle']</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>5</v>
+      </c>
+      <c r="K14" t="n">
+        <v>5</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>motion</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>multihead</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>[{'features': ['wv', 'sv', 'yr', 'ya', 'rarad'], 'output_dim': 4, 'reps': 1, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [0, 1, 2, 3, 4, 0, 1, 2, 3]}]</t>
+        </is>
+      </c>
+      <c r="R14" t="n">
+        <v>1</v>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>compact</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>effsu2</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>lin</t>
+        </is>
+      </c>
+      <c r="V14" t="n">
+        <v>1</v>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>[0, 1, 2, 3, 4, 0, 1, 2, 3]</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>spsa</t>
+        </is>
+      </c>
+      <c r="Z14" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AB14" t="inlineStr"/>
+      <c r="AC14" t="n">
+        <v>512</v>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>[0.05, 0.001]</t>
+        </is>
+      </c>
+      <c r="AE14" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AF14" t="n">
+        <v>130</v>
+      </c>
+      <c r="AG14" t="n">
+        <v>10</v>
+      </c>
+      <c r="AH14" t="n">
+        <v>120</v>
+      </c>
+      <c r="AI14" t="n">
+        <v>0.244048942454759</v>
+      </c>
+      <c r="AJ14" t="n">
+        <v>63.67676614518323</v>
+      </c>
+      <c r="AK14" t="n">
+        <v>0.1214466885563936</v>
+      </c>
+      <c r="AL14" t="n">
+        <v>0.02943226837279816</v>
+      </c>
+      <c r="AM14" t="n">
+        <v>72.52496403951857</v>
+      </c>
+      <c r="AN14" t="n">
+        <v>0.08066171424721016</v>
+      </c>
+      <c r="AO14" t="n">
+        <v>72.52496403951857</v>
+      </c>
+      <c r="AP14" t="n">
+        <v>72.52496403951857</v>
+      </c>
+      <c r="AQ14" t="n">
+        <v>0.08066171424721016</v>
+      </c>
+      <c r="AR14" t="n">
+        <v>101.7254579701999</v>
+      </c>
+      <c r="AS14" t="n">
+        <v>0.0282453306565861</v>
+      </c>
+      <c r="AT14" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AU14" t="inlineStr">
+        <is>
+          <t>identity</t>
+        </is>
+      </c>
+      <c r="AV14" t="n">
+        <v>0.1309183097038825</v>
+      </c>
+      <c r="AW14" t="n">
+        <v>0.04936379960379722</v>
+      </c>
+      <c r="AX14" t="n">
+        <v>0.1309183097038825</v>
+      </c>
+      <c r="AY14" t="n">
+        <v>0.1309183097038825</v>
+      </c>
+      <c r="AZ14" t="n">
+        <v>0.04936379960379722</v>
+      </c>
+      <c r="BA14" t="n">
+        <v>0.1347858431394686</v>
+      </c>
+      <c r="BB14" t="n">
+        <v>0.02128050630107425</v>
+      </c>
+      <c r="BC14" t="n">
+        <v>0.2799409033512636</v>
+      </c>
+      <c r="BD14" t="n">
+        <v>0.03006456022892223</v>
+      </c>
+      <c r="BE14" t="n">
+        <v>0.2799409033512636</v>
+      </c>
+      <c r="BF14" t="n">
+        <v>0.2799409033512636</v>
+      </c>
+      <c r="BG14" t="n">
+        <v>0.03006456022892223</v>
+      </c>
+      <c r="BH14" t="n">
+        <v>0.2546939356941757</v>
+      </c>
+      <c r="BI14" t="n">
+        <v>0.1175399108626123</v>
+      </c>
+      <c r="BJ14" t="n">
+        <v>0.2323811834845038</v>
+      </c>
+      <c r="BK14" t="n">
+        <v>0.06706305092070242</v>
+      </c>
+      <c r="BL14" t="n">
+        <v>0.2323811834845038</v>
+      </c>
+      <c r="BM14" t="n">
+        <v>0.2323811834845038</v>
+      </c>
+      <c r="BN14" t="n">
+        <v>0.06706305092070242</v>
+      </c>
+      <c r="BO14" t="n">
+        <v>0.2165674147770466</v>
+      </c>
+      <c r="BP14" t="n">
+        <v>0.1305503303559786</v>
+      </c>
+      <c r="BQ14" t="n">
+        <v>289.4566157615337</v>
+      </c>
+      <c r="BR14" t="n">
+        <v>0.1761554462354186</v>
+      </c>
+      <c r="BS14" t="n">
+        <v>289.4566157615337</v>
+      </c>
+      <c r="BT14" t="n">
+        <v>289.4566157615337</v>
+      </c>
+      <c r="BU14" t="n">
+        <v>0.1761554462354186</v>
+      </c>
+      <c r="BV14" t="n">
+        <v>406.2957846871897</v>
+      </c>
+      <c r="BW14" t="n">
+        <v>-0.1563894248933255</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>46081.37170138889</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>02-28_08-55-15_multihead_spsa_compact_f5_w5_h5_effsu2_lin_r1.pkl</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Best (Lowest Val Loss)</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>data/reduce_row_number_absolutes</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>16590</v>
+      </c>
+      <c r="G15" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>['wv', 'sv', 'yr', 'ya', 'rarad']</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>['Surge Velocity', 'Sway Velocity', 'Yaw Rate', 'Yaw Angle']</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>5</v>
+      </c>
+      <c r="K15" t="n">
+        <v>5</v>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>motion</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>multihead</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>[{'features': ['wv', 'sv', 'yr', 'ya', 'rarad'], 'output_dim': 4, 'reps': 1, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [0, 1, 2, 3, 4, 0, 1, 2, 3]}]</t>
+        </is>
+      </c>
+      <c r="R15" t="n">
+        <v>1</v>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>compact</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>effsu2</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>lin</t>
+        </is>
+      </c>
+      <c r="V15" t="n">
+        <v>1</v>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>[0, 1, 2, 3, 4, 0, 1, 2, 3]</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>spsa</t>
+        </is>
+      </c>
+      <c r="Z15" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="n">
+        <v>512</v>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>[0.05, 0.001]</t>
+        </is>
+      </c>
+      <c r="AE15" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AF15" t="n">
+        <v>130</v>
+      </c>
+      <c r="AG15" t="n">
+        <v>10</v>
+      </c>
+      <c r="AH15" t="n">
+        <v>120</v>
+      </c>
+      <c r="AI15" t="n">
+        <v>0.2258782497552349</v>
+      </c>
+      <c r="AJ15" t="n">
+        <v>48.03796532937024</v>
+      </c>
+      <c r="AK15" t="n">
+        <v>0.2038061515840728</v>
+      </c>
+      <c r="AL15" t="n">
+        <v>-0.01857917388318911</v>
+      </c>
+      <c r="AM15" t="n">
+        <v>60.04554104870937</v>
+      </c>
+      <c r="AN15" t="n">
+        <v>0.1553095434788727</v>
+      </c>
+      <c r="AO15" t="n">
+        <v>60.04554104870937</v>
+      </c>
+      <c r="AP15" t="n">
+        <v>60.04554104870937</v>
+      </c>
+      <c r="AQ15" t="n">
+        <v>0.1553095434788727</v>
+      </c>
+      <c r="AR15" t="n">
+        <v>136.5913824146042</v>
+      </c>
+      <c r="AS15" t="n">
+        <v>-0.01415633887541282</v>
+      </c>
+      <c r="AT15" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AU15" t="inlineStr">
+        <is>
+          <t>identity</t>
+        </is>
+      </c>
+      <c r="AV15" t="n">
+        <v>0.1247431280571075</v>
+      </c>
+      <c r="AW15" t="n">
+        <v>0.0942036026132036</v>
+      </c>
+      <c r="AX15" t="n">
+        <v>0.1247431280571075</v>
+      </c>
+      <c r="AY15" t="n">
+        <v>0.1247431280571075</v>
+      </c>
+      <c r="AZ15" t="n">
+        <v>0.0942036026132036</v>
+      </c>
+      <c r="BA15" t="n">
+        <v>0.1438975182599111</v>
+      </c>
+      <c r="BB15" t="n">
+        <v>-0.04488203609146013</v>
+      </c>
+      <c r="BC15" t="n">
+        <v>0.2519077702059648</v>
+      </c>
+      <c r="BD15" t="n">
+        <v>0.1271933792044356</v>
+      </c>
+      <c r="BE15" t="n">
+        <v>0.2519077702059648</v>
+      </c>
+      <c r="BF15" t="n">
+        <v>0.2519077702059648</v>
+      </c>
+      <c r="BG15" t="n">
+        <v>0.1271933792044356</v>
+      </c>
+      <c r="BH15" t="n">
+        <v>0.2221313073493235</v>
+      </c>
+      <c r="BI15" t="n">
+        <v>0.2303624632858855</v>
+      </c>
+      <c r="BJ15" t="n">
+        <v>0.2287306101608798</v>
+      </c>
+      <c r="BK15" t="n">
+        <v>0.08171894813175695</v>
+      </c>
+      <c r="BL15" t="n">
+        <v>0.2287306101608798</v>
+      </c>
+      <c r="BM15" t="n">
+        <v>0.2287306101608798</v>
+      </c>
+      <c r="BN15" t="n">
+        <v>0.08171894813175695</v>
+      </c>
+      <c r="BO15" t="n">
+        <v>0.1715161571200728</v>
+      </c>
+      <c r="BP15" t="n">
+        <v>0.3114168800501157</v>
+      </c>
+      <c r="BQ15" t="n">
+        <v>239.5767826864137</v>
+      </c>
+      <c r="BR15" t="n">
+        <v>0.3181222439660961</v>
+      </c>
+      <c r="BS15" t="n">
+        <v>239.5767826864137</v>
+      </c>
+      <c r="BT15" t="n">
+        <v>239.5767826864137</v>
+      </c>
+      <c r="BU15" t="n">
+        <v>0.3181222439660961</v>
+      </c>
+      <c r="BV15" t="n">
+        <v>545.8279846756884</v>
+      </c>
+      <c r="BW15" t="n">
+        <v>-0.553522662746206</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>46081.44099537037</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>02-28_10-35-02_multihead_spsa_compact_f5_w5_h5_effsu2_lin_r1.pkl</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Final (Last Iteration)</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>data/reduce_row_number_absolutes</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>16590</v>
+      </c>
+      <c r="G16" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>['wv', 'sv', 'yr', 'ya', 'rarad']</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>['Surge Velocity', 'Sway Velocity', 'Yaw Rate', 'Yaw Angle']</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>5</v>
+      </c>
+      <c r="K16" t="n">
+        <v>5</v>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>motion</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>multihead</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>[{'features': ['wv', 'sv', 'yr', 'ya', 'rarad'], 'output_dim': 4, 'reps': 1, 'encoding': 'compact', 'ansatz': 'effsu2', 'entangle': 'lin', 'map': [0, 1, 2, 3, 4, 0, 1, 2, 3]}]</t>
+        </is>
+      </c>
+      <c r="R16" t="n">
+        <v>1</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>compact</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>effsu2</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>lin</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>[0, 1, 2, 3, 4, 0, 1, 2, 3]</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>spsa</t>
+        </is>
+      </c>
+      <c r="Z16" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>4000</v>
+      </c>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="n">
+        <v>512</v>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>[0.05, 0.001]</t>
+        </is>
+      </c>
+      <c r="AE16" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>130</v>
+      </c>
+      <c r="AG16" t="n">
+        <v>10</v>
+      </c>
+      <c r="AH16" t="n">
+        <v>120</v>
+      </c>
+      <c r="AI16" t="n">
+        <v>0.2198542356450413</v>
+      </c>
+      <c r="AJ16" t="n">
+        <v>49.00704423609787</v>
+      </c>
+      <c r="AK16" t="n">
+        <v>0.2029416600177747</v>
+      </c>
+      <c r="AL16" t="n">
+        <v>-0.05830465117252812</v>
+      </c>
+      <c r="AM16" t="n">
+        <v>61.07992849757259</v>
+      </c>
+      <c r="AN16" t="n">
+        <v>0.1478411004059185</v>
+      </c>
+      <c r="AO16" t="n">
+        <v>61.07992849757259</v>
+      </c>
+      <c r="AP16" t="n">
+        <v>61.07992849757259</v>
+      </c>
+      <c r="AQ16" t="n">
+        <v>0.1478411004059185</v>
+      </c>
+      <c r="AR16" t="n">
+        <v>135.429816734451</v>
+      </c>
+      <c r="AS16" t="n">
+        <v>-0.06173454641491624</v>
+      </c>
+      <c r="AT16" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AU16" t="inlineStr">
+        <is>
+          <t>identity</t>
+        </is>
+      </c>
+      <c r="AV16" t="n">
+        <v>0.1232063647862272</v>
+      </c>
+      <c r="AW16" t="n">
+        <v>0.105362490930983</v>
+      </c>
+      <c r="AX16" t="n">
+        <v>0.1232063647862272</v>
+      </c>
+      <c r="AY16" t="n">
+        <v>0.1232063647862272</v>
+      </c>
+      <c r="AZ16" t="n">
+        <v>0.105362490930983</v>
+      </c>
+      <c r="BA16" t="n">
+        <v>0.1398599026066967</v>
+      </c>
+      <c r="BB16" t="n">
+        <v>-0.01556372597950073</v>
+      </c>
+      <c r="BC16" t="n">
+        <v>0.256061123182084</v>
+      </c>
+      <c r="BD16" t="n">
+        <v>0.112802898223663</v>
+      </c>
+      <c r="BE16" t="n">
+        <v>0.256061123182084</v>
+      </c>
+      <c r="BF16" t="n">
+        <v>0.256061123182084</v>
+      </c>
+      <c r="BG16" t="n">
+        <v>0.112802898223663</v>
+      </c>
+      <c r="BH16" t="n">
+        <v>0.2431533622963736</v>
+      </c>
+      <c r="BI16" t="n">
+        <v>0.1575255328271241</v>
+      </c>
+      <c r="BJ16" t="n">
+        <v>0.2324379962999909</v>
+      </c>
+      <c r="BK16" t="n">
+        <v>0.06683496543652367</v>
+      </c>
+      <c r="BL16" t="n">
+        <v>0.2324379962999909</v>
+      </c>
+      <c r="BM16" t="n">
+        <v>0.2324379962999909</v>
+      </c>
+      <c r="BN16" t="n">
+        <v>0.06683496543652367</v>
+      </c>
+      <c r="BO16" t="n">
+        <v>0.2114147403486813</v>
+      </c>
+      <c r="BP16" t="n">
+        <v>0.1512366883851284</v>
+      </c>
+      <c r="BQ16" t="n">
+        <v>243.7080085060227</v>
+      </c>
+      <c r="BR16" t="n">
+        <v>0.3063640470324994</v>
+      </c>
+      <c r="BS16" t="n">
+        <v>243.7080085060227</v>
+      </c>
+      <c r="BT16" t="n">
+        <v>243.7080085060227</v>
+      </c>
+      <c r="BU16" t="n">
+        <v>0.3063640470324994</v>
+      </c>
+      <c r="BV16" t="n">
+        <v>541.1248389325534</v>
+      </c>
+      <c r="BW16" t="n">
+        <v>-0.5401366808924177</v>
       </c>
     </row>
   </sheetData>

</xml_diff>